<commit_message>
keeping original comp weights for testing
</commit_message>
<xml_diff>
--- a/Data/GOA_25.1.1_arrowtooth_single_species_1977-2024.xlsx
+++ b/Data/GOA_25.1.1_arrowtooth_single_species_1977-2024.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kalei.shotwell\Work\GitHub\GOA-ATF-ESP\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE0E561-0DE4-49DE-9705-929133932FB1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F5812CF-00EE-4C05-9AD7-DE41D52D1286}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="12" windowWidth="16092" windowHeight="9660" firstSheet="4" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="12" windowWidth="16092" windowHeight="9660" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="meta_data" sheetId="1" r:id="rId1"/>
@@ -57439,7 +57439,7 @@
         <v>0</v>
       </c>
       <c r="AA2">
-        <v>1</v>
+        <v>0.1188226</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
@@ -57504,7 +57504,7 @@
         <v>0</v>
       </c>
       <c r="AA3">
-        <v>1</v>
+        <v>0.1173554</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
@@ -57551,7 +57551,7 @@
         <v>0</v>
       </c>
       <c r="AA4">
-        <v>1</v>
+        <v>0.10607419999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>